<commit_message>
Fix phone-dedup case in contacts exercise data
Иван Иванов previously shared the same email (ivanov@mail.ru) across both
the webinar and CRM exports, so a dedup-by-email-only agent would merge his
records without ever using phone normalization. Changed his CRM email to a
distinct (stale corporate) address so the two records now link ONLY by phone
in different formats — matching what 260-cowork/self_study.md claims the case
teaches.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/documents/контакты/Клиенты CRM.xlsx
+++ b/documents/контакты/Клиенты CRM.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Клиенты" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Клиенты" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -446,7 +446,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ivanov@mail.ru</t>
+          <t>i.ivanov@old-corp.ru</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -520,7 +520,6 @@
           <t>89123334708</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">

</xml_diff>